<commit_message>
did monthly revision and made some chnages
</commit_message>
<xml_diff>
--- a/introduction.xlsx
+++ b/introduction.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code-fun\EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5231EC63-FB04-4E92-B46E-AD54F033ACD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214B9A2A-35FE-41A9-AD87-97E87E0D4CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="470">
   <si>
     <t>DATA FOLDER IN RIBBON ALLOWS TO IMPORT DATA</t>
   </si>
@@ -1934,6 +1934,12 @@
       </rPr>
       <t xml:space="preserve"> press krna h</t>
     </r>
+  </si>
+  <si>
+    <t>exact match: excat value do</t>
+  </si>
+  <si>
+    <t>approximate match: "If you can't find it, give me the nearest lower value."</t>
   </si>
 </sst>
 </file>
@@ -2278,6 +2284,12 @@
     <xf numFmtId="165" fontId="0" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2308,45 +2320,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="45">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color theme="5"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="42">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2787,24 +2767,24 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{C13D1EE1-26BC-4064-A6EC-56C85878DF7D}" name="Table13" displayName="Table13" ref="B231:E246" totalsRowShown="0" headerRowDxfId="33" headerRowBorderDxfId="32" tableBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{C13D1EE1-26BC-4064-A6EC-56C85878DF7D}" name="Table13" displayName="Table13" ref="B231:E246" totalsRowShown="0" headerRowDxfId="30" headerRowBorderDxfId="29" tableBorderDxfId="28">
   <autoFilter ref="B231:E246" xr:uid="{C13D1EE1-26BC-4064-A6EC-56C85878DF7D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A11D603B-2DB4-4B99-993A-03CA088269A1}" name="FULL NAME" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{E6FE1425-5580-413E-B00A-BD05EC1CE044}" name="AGE" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{7470512B-6575-400E-8DCB-DC4C94E5625C}" name="GENDER" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{92DCE196-3117-4F0C-915D-CCE17F739272}" name="SALARY" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{A11D603B-2DB4-4B99-993A-03CA088269A1}" name="FULL NAME" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{E6FE1425-5580-413E-B00A-BD05EC1CE044}" name="AGE" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{7470512B-6575-400E-8DCB-DC4C94E5625C}" name="GENDER" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{92DCE196-3117-4F0C-915D-CCE17F739272}" name="SALARY" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{3E81880B-F57F-4375-9CB3-E928E4ECB80A}" name="Table12" displayName="Table12" ref="I461:J465" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{3E81880B-F57F-4375-9CB3-E928E4ECB80A}" name="Table12" displayName="Table12" ref="I461:J465" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="I461:J465" xr:uid="{3E81880B-F57F-4375-9CB3-E928E4ECB80A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{BB6CC05A-A401-4107-8F61-333D82A6D853}" name="country" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{80A488B2-0ABE-418B-8F19-B4D5F306B9B5}" name="COUNTRY_via_lookup" dataDxfId="23">
+    <tableColumn id="1" xr3:uid="{BB6CC05A-A401-4107-8F61-333D82A6D853}" name="country" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{80A488B2-0ABE-418B-8F19-B4D5F306B9B5}" name="COUNTRY_via_lookup" dataDxfId="20">
       <calculatedColumnFormula>LOOKUP(I462,$L$461:$L$464,$M$461)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2816,14 +2796,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Table_1" displayName="Table_1" ref="A1:H10" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
   <tableColumns count="8">
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0900-000011000000}" uniqueName="17" name="Time" queryTableFieldId="1" dataDxfId="22"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0900-000012000000}" uniqueName="18" name="Cur." queryTableFieldId="2" dataDxfId="21"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0900-000013000000}" uniqueName="19" name="Event" queryTableFieldId="3" dataDxfId="20"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0900-000014000000}" uniqueName="20" name="Imp." queryTableFieldId="4" dataDxfId="19"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0900-000015000000}" uniqueName="21" name="Actual" queryTableFieldId="5" dataDxfId="18"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0900-000016000000}" uniqueName="22" name="Forecast" queryTableFieldId="6" dataDxfId="17"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0900-000017000000}" uniqueName="23" name="Previous" queryTableFieldId="7" dataDxfId="16"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0900-000018000000}" uniqueName="24" name="Column8" queryTableFieldId="8" dataDxfId="15"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0900-000011000000}" uniqueName="17" name="Time" queryTableFieldId="1" dataDxfId="19"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0900-000012000000}" uniqueName="18" name="Cur." queryTableFieldId="2" dataDxfId="18"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0900-000013000000}" uniqueName="19" name="Event" queryTableFieldId="3" dataDxfId="17"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0900-000014000000}" uniqueName="20" name="Imp." queryTableFieldId="4" dataDxfId="16"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0900-000015000000}" uniqueName="21" name="Actual" queryTableFieldId="5" dataDxfId="15"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0900-000016000000}" uniqueName="22" name="Forecast" queryTableFieldId="6" dataDxfId="14"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0900-000017000000}" uniqueName="23" name="Previous" queryTableFieldId="7" dataDxfId="13"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0900-000018000000}" uniqueName="24" name="Column8" queryTableFieldId="8" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2833,13 +2813,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="Table_0__2" displayName="Table_0__2" ref="A1:G11" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="7">
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" uniqueName="15" name="Name" queryTableFieldId="1" dataDxfId="14"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" uniqueName="16" name="Last" queryTableFieldId="2" dataDxfId="13"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" uniqueName="17" name="High" queryTableFieldId="3" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" uniqueName="18" name="Low" queryTableFieldId="4" dataDxfId="11"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" uniqueName="19" name="Chg." queryTableFieldId="5" dataDxfId="10"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" uniqueName="20" name="Chg. %" queryTableFieldId="6" dataDxfId="9"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" uniqueName="21" name="Time" queryTableFieldId="7" dataDxfId="8"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" uniqueName="15" name="Name" queryTableFieldId="1" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" uniqueName="16" name="Last" queryTableFieldId="2" dataDxfId="10"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" uniqueName="17" name="High" queryTableFieldId="3" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" uniqueName="18" name="Low" queryTableFieldId="4" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" uniqueName="19" name="Chg." queryTableFieldId="5" dataDxfId="7"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" uniqueName="20" name="Chg. %" queryTableFieldId="6" dataDxfId="6"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" uniqueName="21" name="Time" queryTableFieldId="7" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2849,7 +2829,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table4" displayName="Table4" ref="B78:F82" totalsRowShown="0">
   <autoFilter ref="B78:F82" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="DATE" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="DATE" dataDxfId="41"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="category"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="sub-category"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="amount"/>
@@ -2874,14 +2854,14 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table424" displayName="Table424" ref="B179:F187" totalsRowShown="0" headerRowDxfId="43" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table424" displayName="Table424" ref="B179:F187" totalsRowShown="0" headerRowDxfId="40" dataCellStyle="Normal">
   <autoFilter ref="B179:F187" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="DATE" dataDxfId="42" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="category" dataDxfId="41" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="sub-category" dataDxfId="40" dataCellStyle="Percent"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="amount" dataDxfId="39" dataCellStyle="Percent"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="payment-mode" dataDxfId="38" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="DATE" dataDxfId="39" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="category" dataDxfId="38" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="sub-category" dataDxfId="37" dataCellStyle="Percent"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="amount" dataDxfId="36" dataCellStyle="Percent"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="payment-mode" dataDxfId="35" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2892,21 +2872,21 @@
   <autoFilter ref="B200:E215" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B201:E215">
     <sortCondition descending="1" ref="C201:C215"/>
-    <sortCondition descending="1" ref="E201:E215"/>
+    <sortCondition ref="D201:D215"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="DATE" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="DATE" dataDxfId="34"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="CATEGORY"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SUB-CATEGORY"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="AMOUNT" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="AMOUNT" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table6" displayName="Table6" ref="B275:E281" totalsRowShown="0">
-  <autoFilter ref="B275:E281" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table6" displayName="Table6" ref="B275:E280" totalsRowShown="0">
+  <autoFilter ref="B275:E280" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="name"/>
@@ -2921,10 +2901,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Table510" displayName="Table510" ref="B414:E429" totalsRowShown="0">
   <autoFilter ref="B414:E429" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="DATE" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="DATE" dataDxfId="32"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="CATEGORY"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="SUB-CATEGORY"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="AMOUNT" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="AMOUNT" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3270,60 +3250,60 @@
       <c r="H8" s="3"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9" s="47" t="s">
+      <c r="A9" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="47"/>
-      <c r="C9" s="47"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="47"/>
-      <c r="F9" s="47"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="47"/>
-      <c r="I9" s="47"/>
-      <c r="J9" s="47"/>
-      <c r="K9" s="47"/>
-      <c r="L9" s="47"/>
-      <c r="M9" s="47"/>
-      <c r="N9" s="47"/>
-      <c r="O9" s="47"/>
-      <c r="P9" s="47"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="49"/>
+      <c r="L9" s="49"/>
+      <c r="M9" s="49"/>
+      <c r="N9" s="49"/>
+      <c r="O9" s="49"/>
+      <c r="P9" s="49"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A10" s="47"/>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="47"/>
-      <c r="L10" s="47"/>
-      <c r="M10" s="47"/>
-      <c r="N10" s="47"/>
-      <c r="O10" s="47"/>
-      <c r="P10" s="47"/>
+      <c r="A10" s="49"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
+      <c r="N10" s="49"/>
+      <c r="O10" s="49"/>
+      <c r="P10" s="49"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A11" s="47"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="47"/>
-      <c r="P11" s="47"/>
+      <c r="A11" s="49"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="49"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49"/>
+      <c r="M11" s="49"/>
+      <c r="N11" s="49"/>
+      <c r="O11" s="49"/>
+      <c r="P11" s="49"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -3334,14 +3314,14 @@
       <c r="A14" t="s">
         <v>5</v>
       </c>
-      <c r="I14" s="54"/>
-      <c r="J14" s="54"/>
+      <c r="I14" s="56"/>
+      <c r="J14" s="56"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="E15" s="57"/>
-      <c r="F15" s="57"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="54"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
+      <c r="I15" s="56"/>
+      <c r="J15" s="56"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
@@ -3349,8 +3329,8 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
-      <c r="E16" s="57"/>
-      <c r="F16" s="57"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -3428,66 +3408,66 @@
       </c>
     </row>
     <row r="25" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="48" t="s">
+      <c r="B25" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="49"/>
-      <c r="J25" s="49"/>
-      <c r="K25" s="49"/>
-      <c r="L25" s="49"/>
-      <c r="M25" s="49"/>
-      <c r="N25" s="49"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="51"/>
+      <c r="E25" s="51"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="51"/>
+      <c r="H25" s="51"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="51"/>
+      <c r="K25" s="51"/>
+      <c r="L25" s="51"/>
+      <c r="M25" s="51"/>
+      <c r="N25" s="51"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B26" s="49"/>
-      <c r="C26" s="49"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="49"/>
-      <c r="K26" s="49"/>
-      <c r="L26" s="49"/>
-      <c r="M26" s="49"/>
-      <c r="N26" s="49"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="51"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B27" s="49"/>
-      <c r="C27" s="49"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="49"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="49"/>
-      <c r="M27" s="49"/>
-      <c r="N27" s="49"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="51"/>
+      <c r="L27" s="51"/>
+      <c r="M27" s="51"/>
+      <c r="N27" s="51"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B28" s="49"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="49"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="49"/>
-      <c r="H28" s="49"/>
-      <c r="I28" s="49"/>
-      <c r="J28" s="49"/>
-      <c r="K28" s="49"/>
-      <c r="L28" s="49"/>
-      <c r="M28" s="49"/>
-      <c r="N28" s="49"/>
+      <c r="B28" s="51"/>
+      <c r="C28" s="51"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="51"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="51"/>
+      <c r="K28" s="51"/>
+      <c r="L28" s="51"/>
+      <c r="M28" s="51"/>
+      <c r="N28" s="51"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
@@ -3709,45 +3689,45 @@
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B72" s="50" t="s">
+      <c r="B72" s="52" t="s">
         <v>54</v>
       </c>
-      <c r="C72" s="49"/>
-      <c r="D72" s="49"/>
-      <c r="E72" s="49"/>
-      <c r="F72" s="49"/>
-      <c r="G72" s="49"/>
-      <c r="H72" s="49"/>
-      <c r="I72" s="49"/>
-      <c r="J72" s="49"/>
-      <c r="K72" s="49"/>
-      <c r="L72" s="49"/>
+      <c r="C72" s="51"/>
+      <c r="D72" s="51"/>
+      <c r="E72" s="51"/>
+      <c r="F72" s="51"/>
+      <c r="G72" s="51"/>
+      <c r="H72" s="51"/>
+      <c r="I72" s="51"/>
+      <c r="J72" s="51"/>
+      <c r="K72" s="51"/>
+      <c r="L72" s="51"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B73" s="49"/>
-      <c r="C73" s="49"/>
-      <c r="D73" s="49"/>
-      <c r="E73" s="49"/>
-      <c r="F73" s="49"/>
-      <c r="G73" s="49"/>
-      <c r="H73" s="49"/>
-      <c r="I73" s="49"/>
-      <c r="J73" s="49"/>
-      <c r="K73" s="49"/>
-      <c r="L73" s="49"/>
+      <c r="B73" s="51"/>
+      <c r="C73" s="51"/>
+      <c r="D73" s="51"/>
+      <c r="E73" s="51"/>
+      <c r="F73" s="51"/>
+      <c r="G73" s="51"/>
+      <c r="H73" s="51"/>
+      <c r="I73" s="51"/>
+      <c r="J73" s="51"/>
+      <c r="K73" s="51"/>
+      <c r="L73" s="51"/>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B74" s="49"/>
-      <c r="C74" s="49"/>
-      <c r="D74" s="49"/>
-      <c r="E74" s="49"/>
-      <c r="F74" s="49"/>
-      <c r="G74" s="49"/>
-      <c r="H74" s="49"/>
-      <c r="I74" s="49"/>
-      <c r="J74" s="49"/>
-      <c r="K74" s="49"/>
-      <c r="L74" s="49"/>
+      <c r="B74" s="51"/>
+      <c r="C74" s="51"/>
+      <c r="D74" s="51"/>
+      <c r="E74" s="51"/>
+      <c r="F74" s="51"/>
+      <c r="G74" s="51"/>
+      <c r="H74" s="51"/>
+      <c r="I74" s="51"/>
+      <c r="J74" s="51"/>
+      <c r="K74" s="51"/>
+      <c r="L74" s="51"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
@@ -3881,33 +3861,33 @@
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B98" s="51" t="s">
+      <c r="B98" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="C98" s="52"/>
-      <c r="D98" s="52"/>
-      <c r="E98" s="52"/>
-      <c r="F98" s="52"/>
-      <c r="G98" s="52"/>
-      <c r="H98" s="52"/>
+      <c r="C98" s="54"/>
+      <c r="D98" s="54"/>
+      <c r="E98" s="54"/>
+      <c r="F98" s="54"/>
+      <c r="G98" s="54"/>
+      <c r="H98" s="54"/>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B99" s="52"/>
-      <c r="C99" s="52"/>
-      <c r="D99" s="52"/>
-      <c r="E99" s="52"/>
-      <c r="F99" s="52"/>
-      <c r="G99" s="52"/>
-      <c r="H99" s="52"/>
+      <c r="B99" s="54"/>
+      <c r="C99" s="54"/>
+      <c r="D99" s="54"/>
+      <c r="E99" s="54"/>
+      <c r="F99" s="54"/>
+      <c r="G99" s="54"/>
+      <c r="H99" s="54"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B100" s="52"/>
-      <c r="C100" s="52"/>
-      <c r="D100" s="52"/>
-      <c r="E100" s="52"/>
-      <c r="F100" s="52"/>
-      <c r="G100" s="52"/>
-      <c r="H100" s="52"/>
+      <c r="B100" s="54"/>
+      <c r="C100" s="54"/>
+      <c r="D100" s="54"/>
+      <c r="E100" s="54"/>
+      <c r="F100" s="54"/>
+      <c r="G100" s="54"/>
+      <c r="H100" s="54"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
@@ -4174,7 +4154,7 @@
       <c r="B138" s="9">
         <v>1</v>
       </c>
-      <c r="D138" s="58">
+      <c r="D138">
         <v>54</v>
       </c>
       <c r="E138" s="34" t="s">
@@ -4188,7 +4168,7 @@
       <c r="B139" s="9">
         <v>2</v>
       </c>
-      <c r="D139" s="58">
+      <c r="D139">
         <v>65</v>
       </c>
       <c r="E139" s="34" t="s">
@@ -4202,7 +4182,7 @@
       <c r="B140" s="9">
         <v>3</v>
       </c>
-      <c r="D140" s="58">
+      <c r="D140">
         <v>32</v>
       </c>
       <c r="E140" s="34" t="s">
@@ -4216,7 +4196,7 @@
       <c r="B141" s="9">
         <v>4</v>
       </c>
-      <c r="D141" s="58">
+      <c r="D141">
         <v>45</v>
       </c>
       <c r="E141" s="34" t="s">
@@ -4230,7 +4210,7 @@
       <c r="B142" s="9">
         <v>5</v>
       </c>
-      <c r="D142" s="58">
+      <c r="D142">
         <v>21</v>
       </c>
     </row>
@@ -4238,7 +4218,7 @@
       <c r="B143" s="9">
         <v>6</v>
       </c>
-      <c r="D143" s="58">
+      <c r="D143">
         <v>55</v>
       </c>
     </row>
@@ -4246,7 +4226,7 @@
       <c r="B144" s="9">
         <v>7</v>
       </c>
-      <c r="D144" s="58">
+      <c r="D144">
         <v>0</v>
       </c>
     </row>
@@ -4254,7 +4234,7 @@
       <c r="B145" s="9">
         <v>8</v>
       </c>
-      <c r="D145" s="58">
+      <c r="D145">
         <v>100</v>
       </c>
     </row>
@@ -4262,7 +4242,7 @@
       <c r="B146" s="9">
         <v>9</v>
       </c>
-      <c r="D146" s="58">
+      <c r="D146">
         <v>54</v>
       </c>
     </row>
@@ -4354,34 +4334,34 @@
       </c>
     </row>
     <row r="163" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B163" s="53" t="s">
+      <c r="B163" s="55" t="s">
         <v>94</v>
       </c>
-      <c r="C163" s="52"/>
-      <c r="D163" s="52"/>
-      <c r="E163" s="52"/>
-      <c r="F163" s="52"/>
+      <c r="C163" s="54"/>
+      <c r="D163" s="54"/>
+      <c r="E163" s="54"/>
+      <c r="F163" s="54"/>
     </row>
     <row r="164" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B164" s="52"/>
-      <c r="C164" s="52"/>
-      <c r="D164" s="52"/>
-      <c r="E164" s="52"/>
-      <c r="F164" s="52"/>
+      <c r="B164" s="54"/>
+      <c r="C164" s="54"/>
+      <c r="D164" s="54"/>
+      <c r="E164" s="54"/>
+      <c r="F164" s="54"/>
     </row>
     <row r="165" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B165" s="52"/>
-      <c r="C165" s="52"/>
-      <c r="D165" s="52"/>
-      <c r="E165" s="52"/>
-      <c r="F165" s="52"/>
+      <c r="B165" s="54"/>
+      <c r="C165" s="54"/>
+      <c r="D165" s="54"/>
+      <c r="E165" s="54"/>
+      <c r="F165" s="54"/>
     </row>
     <row r="166" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B166" s="52"/>
-      <c r="C166" s="52"/>
-      <c r="D166" s="52"/>
-      <c r="E166" s="52"/>
-      <c r="F166" s="52"/>
+      <c r="B166" s="54"/>
+      <c r="C166" s="54"/>
+      <c r="D166" s="54"/>
+      <c r="E166" s="54"/>
+      <c r="F166" s="54"/>
     </row>
     <row r="168" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B168" s="10">
@@ -4405,32 +4385,32 @@
       </c>
     </row>
     <row r="171" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B171">
+      <c r="B171" s="48">
         <v>45</v>
       </c>
     </row>
     <row r="172" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B172">
+      <c r="B172" s="48">
         <v>21</v>
       </c>
     </row>
     <row r="173" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B173">
+      <c r="B173" s="48">
         <v>55</v>
       </c>
     </row>
     <row r="174" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B174">
+      <c r="B174" s="48">
         <v>0</v>
       </c>
     </row>
     <row r="175" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B175">
+      <c r="B175" s="48">
         <v>100</v>
       </c>
     </row>
     <row r="176" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B176">
+      <c r="B176" s="48">
         <v>54</v>
       </c>
     </row>
@@ -4608,34 +4588,34 @@
       </c>
     </row>
     <row r="194" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B194" s="51" t="s">
+      <c r="B194" s="53" t="s">
         <v>124</v>
       </c>
-      <c r="C194" s="52"/>
-      <c r="D194" s="52"/>
-      <c r="E194" s="52"/>
-      <c r="F194" s="52"/>
+      <c r="C194" s="54"/>
+      <c r="D194" s="54"/>
+      <c r="E194" s="54"/>
+      <c r="F194" s="54"/>
     </row>
     <row r="195" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B195" s="52"/>
-      <c r="C195" s="52"/>
-      <c r="D195" s="52"/>
-      <c r="E195" s="52"/>
-      <c r="F195" s="52"/>
+      <c r="B195" s="54"/>
+      <c r="C195" s="54"/>
+      <c r="D195" s="54"/>
+      <c r="E195" s="54"/>
+      <c r="F195" s="54"/>
     </row>
     <row r="196" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B196" s="52"/>
-      <c r="C196" s="52"/>
-      <c r="D196" s="52"/>
-      <c r="E196" s="52"/>
-      <c r="F196" s="52"/>
+      <c r="B196" s="54"/>
+      <c r="C196" s="54"/>
+      <c r="D196" s="54"/>
+      <c r="E196" s="54"/>
+      <c r="F196" s="54"/>
     </row>
     <row r="197" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B197" s="52"/>
-      <c r="C197" s="52"/>
-      <c r="D197" s="52"/>
-      <c r="E197" s="52"/>
-      <c r="F197" s="52"/>
+      <c r="B197" s="54"/>
+      <c r="C197" s="54"/>
+      <c r="D197" s="54"/>
+      <c r="E197" s="54"/>
+      <c r="F197" s="54"/>
     </row>
     <row r="199" spans="2:13" x14ac:dyDescent="0.35">
       <c r="C199" t="s">
@@ -4937,34 +4917,34 @@
       </c>
     </row>
     <row r="226" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B226" s="51" t="s">
+      <c r="B226" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="C226" s="52"/>
-      <c r="D226" s="52"/>
-      <c r="E226" s="52"/>
-      <c r="F226" s="52"/>
+      <c r="C226" s="54"/>
+      <c r="D226" s="54"/>
+      <c r="E226" s="54"/>
+      <c r="F226" s="54"/>
     </row>
     <row r="227" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B227" s="52"/>
-      <c r="C227" s="52"/>
-      <c r="D227" s="52"/>
-      <c r="E227" s="52"/>
-      <c r="F227" s="52"/>
+      <c r="B227" s="54"/>
+      <c r="C227" s="54"/>
+      <c r="D227" s="54"/>
+      <c r="E227" s="54"/>
+      <c r="F227" s="54"/>
     </row>
     <row r="228" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B228" s="52"/>
-      <c r="C228" s="52"/>
-      <c r="D228" s="52"/>
-      <c r="E228" s="52"/>
-      <c r="F228" s="52"/>
+      <c r="B228" s="54"/>
+      <c r="C228" s="54"/>
+      <c r="D228" s="54"/>
+      <c r="E228" s="54"/>
+      <c r="F228" s="54"/>
     </row>
     <row r="229" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B229" s="52"/>
-      <c r="C229" s="52"/>
-      <c r="D229" s="52"/>
-      <c r="E229" s="52"/>
-      <c r="F229" s="52"/>
+      <c r="B229" s="54"/>
+      <c r="C229" s="54"/>
+      <c r="D229" s="54"/>
+      <c r="E229" s="54"/>
+      <c r="F229" s="54"/>
     </row>
     <row r="231" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B231" s="40" t="s">
@@ -4985,7 +4965,8 @@
         <v>134</v>
       </c>
       <c r="C232" s="15">
-        <v>23</v>
+        <f>I231</f>
+        <v>0</v>
       </c>
       <c r="D232" s="15" t="s">
         <v>13</v>
@@ -4999,8 +4980,8 @@
         <v>135</v>
       </c>
       <c r="C233" s="16">
-        <f>C232</f>
-        <v>23</v>
+        <f>G232</f>
+        <v>0</v>
       </c>
       <c r="D233" s="16" t="str">
         <f>D232</f>
@@ -5023,30 +5004,29 @@
       <c r="E234" s="18">
         <v>533423</v>
       </c>
+      <c r="G234">
+        <f>AVERAGE(Table13[SALARY])</f>
+        <v>140907.5</v>
+      </c>
     </row>
     <row r="235" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B235" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="C235" s="16">
-        <f>C234</f>
-        <v>103.9</v>
-      </c>
+      <c r="C235" s="16"/>
       <c r="D235" s="16" t="str">
         <f>D234</f>
         <v>M</v>
       </c>
       <c r="E235" s="19">
-        <v>65425</v>
+        <v>140907.5</v>
       </c>
     </row>
     <row r="236" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B236" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="C236" s="15">
-        <v>103.9</v>
-      </c>
+      <c r="C236" s="15"/>
       <c r="D236" s="15" t="s">
         <v>13</v>
       </c>
@@ -5065,12 +5045,9 @@
         <v>140</v>
       </c>
       <c r="E237" s="19">
-        <v>122628</v>
-      </c>
-      <c r="F237" s="17">
-        <f>AVERAGE(E232:E246)</f>
-        <v>122628.2</v>
-      </c>
+        <v>140907.5</v>
+      </c>
+      <c r="F237" s="17"/>
     </row>
     <row r="238" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B238" s="38" t="s">
@@ -5092,26 +5069,21 @@
         <v>134</v>
       </c>
       <c r="C239" s="15">
-        <v>23</v>
+        <f>I238</f>
+        <v>0</v>
       </c>
       <c r="D239" s="15" t="s">
         <v>13</v>
       </c>
       <c r="E239" s="18">
-        <v>54242</v>
-      </c>
-      <c r="F239">
-        <f>AVERAGE(Table13[SALARY])</f>
-        <v>122628.2</v>
+        <v>140907.5</v>
       </c>
     </row>
     <row r="240" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B240" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="C240" s="16">
-        <v>103.9</v>
-      </c>
+      <c r="C240" s="16"/>
       <c r="D240" s="16" t="str">
         <f>D239</f>
         <v>F</v>
@@ -5119,17 +5091,14 @@
       <c r="E240" s="19">
         <v>137814</v>
       </c>
-      <c r="G240">
-        <f>AVERAGE(Table13[AGE])</f>
-        <v>100.96666666666667</v>
-      </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B241" s="38" t="s">
         <v>136</v>
       </c>
       <c r="C241" s="15">
-        <v>21</v>
+        <f>I240</f>
+        <v>0</v>
       </c>
       <c r="D241" s="15" t="s">
         <v>140</v>
@@ -5143,15 +5112,15 @@
         <v>137</v>
       </c>
       <c r="C242" s="16">
-        <f>C241</f>
-        <v>21</v>
+        <f t="shared" ref="C242:C243" si="0">G241</f>
+        <v>0</v>
       </c>
       <c r="D242" s="16" t="str">
         <f>D241</f>
         <v>M</v>
       </c>
       <c r="E242" s="19">
-        <v>65425</v>
+        <v>140907.5</v>
       </c>
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.35">
@@ -5159,7 +5128,8 @@
         <v>29</v>
       </c>
       <c r="C243" s="15">
-        <v>763</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D243" s="15" t="s">
         <v>13</v>
@@ -5179,7 +5149,7 @@
         <v>140</v>
       </c>
       <c r="E244" s="19">
-        <v>122628</v>
+        <v>140907.5</v>
       </c>
     </row>
     <row r="245" spans="1:5" x14ac:dyDescent="0.35">
@@ -5187,7 +5157,8 @@
         <v>139</v>
       </c>
       <c r="C245" s="15">
-        <v>54</v>
+        <f>C246</f>
+        <v>23</v>
       </c>
       <c r="D245" s="15" t="s">
         <v>13</v>
@@ -5280,30 +5251,30 @@
       </c>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B265" s="51" t="s">
+      <c r="B265" s="53" t="s">
         <v>156</v>
       </c>
-      <c r="C265" s="52"/>
-      <c r="D265" s="52"/>
-      <c r="E265" s="52"/>
+      <c r="C265" s="54"/>
+      <c r="D265" s="54"/>
+      <c r="E265" s="54"/>
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B266" s="52"/>
-      <c r="C266" s="52"/>
-      <c r="D266" s="52"/>
-      <c r="E266" s="52"/>
+      <c r="B266" s="54"/>
+      <c r="C266" s="54"/>
+      <c r="D266" s="54"/>
+      <c r="E266" s="54"/>
     </row>
     <row r="267" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B267" s="52"/>
-      <c r="C267" s="52"/>
-      <c r="D267" s="52"/>
-      <c r="E267" s="52"/>
+      <c r="B267" s="54"/>
+      <c r="C267" s="54"/>
+      <c r="D267" s="54"/>
+      <c r="E267" s="54"/>
     </row>
     <row r="268" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B268" s="52"/>
-      <c r="C268" s="52"/>
-      <c r="D268" s="52"/>
-      <c r="E268" s="52"/>
+      <c r="B268" s="54"/>
+      <c r="C268" s="54"/>
+      <c r="D268" s="54"/>
+      <c r="E268" s="54"/>
     </row>
     <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B270" t="s">
@@ -5408,18 +5379,6 @@
       </c>
     </row>
     <row r="280" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B280">
-        <v>8</v>
-      </c>
-      <c r="C280" t="s">
-        <v>12</v>
-      </c>
-      <c r="D280">
-        <v>44</v>
-      </c>
-      <c r="E280" t="s">
-        <v>13</v>
-      </c>
       <c r="G280" t="s">
         <v>167</v>
       </c>
@@ -5435,30 +5394,30 @@
       </c>
     </row>
     <row r="283" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B283" s="50" t="s">
+      <c r="B283" s="52" t="s">
         <v>169</v>
       </c>
-      <c r="C283" s="49"/>
-      <c r="D283" s="49"/>
-      <c r="E283" s="49"/>
+      <c r="C283" s="51"/>
+      <c r="D283" s="51"/>
+      <c r="E283" s="51"/>
     </row>
     <row r="284" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B284" s="49"/>
-      <c r="C284" s="49"/>
-      <c r="D284" s="49"/>
-      <c r="E284" s="49"/>
+      <c r="B284" s="51"/>
+      <c r="C284" s="51"/>
+      <c r="D284" s="51"/>
+      <c r="E284" s="51"/>
     </row>
     <row r="285" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B285" s="49"/>
-      <c r="C285" s="49"/>
-      <c r="D285" s="49"/>
-      <c r="E285" s="49"/>
+      <c r="B285" s="51"/>
+      <c r="C285" s="51"/>
+      <c r="D285" s="51"/>
+      <c r="E285" s="51"/>
     </row>
     <row r="286" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B286" s="49"/>
-      <c r="C286" s="49"/>
-      <c r="D286" s="49"/>
-      <c r="E286" s="49"/>
+      <c r="B286" s="51"/>
+      <c r="C286" s="51"/>
+      <c r="D286" s="51"/>
+      <c r="E286" s="51"/>
     </row>
     <row r="288" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B288" t="s">
@@ -5489,7 +5448,7 @@
         <v>173</v>
       </c>
       <c r="C293" t="str">
-        <f t="shared" ref="C293:C295" si="0">TRIM(B293)</f>
+        <f t="shared" ref="C293:C295" si="1">TRIM(B293)</f>
         <v>IMAN</v>
       </c>
     </row>
@@ -5498,7 +5457,7 @@
         <v>174</v>
       </c>
       <c r="C294" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>KOSAM</v>
       </c>
     </row>
@@ -5507,29 +5466,29 @@
         <v>175</v>
       </c>
       <c r="C295" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>SULTAN</v>
       </c>
     </row>
     <row r="297" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B297" s="50" t="s">
+      <c r="B297" s="52" t="s">
         <v>177</v>
       </c>
-      <c r="C297" s="49"/>
-      <c r="D297" s="49"/>
-      <c r="E297" s="49"/>
+      <c r="C297" s="51"/>
+      <c r="D297" s="51"/>
+      <c r="E297" s="51"/>
     </row>
     <row r="298" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B298" s="49"/>
-      <c r="C298" s="49"/>
-      <c r="D298" s="49"/>
-      <c r="E298" s="49"/>
+      <c r="B298" s="51"/>
+      <c r="C298" s="51"/>
+      <c r="D298" s="51"/>
+      <c r="E298" s="51"/>
     </row>
     <row r="299" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B299" s="49"/>
-      <c r="C299" s="49"/>
-      <c r="D299" s="49"/>
-      <c r="E299" s="49"/>
+      <c r="B299" s="51"/>
+      <c r="C299" s="51"/>
+      <c r="D299" s="51"/>
+      <c r="E299" s="51"/>
     </row>
     <row r="301" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B301" t="s">
@@ -5695,6 +5654,14 @@
         <f>REPLACE(B339,1,3,"new")</f>
         <v>new text</v>
       </c>
+      <c r="D339" t="str">
+        <f>REPLACE(B339,1,3,"ok")</f>
+        <v>ok text</v>
+      </c>
+      <c r="F339" t="str">
+        <f>REPLACE(B339,1,4,"n")</f>
+        <v>ntext</v>
+      </c>
     </row>
     <row r="340" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C340" t="str">
@@ -5714,7 +5681,7 @@
         <v>442</v>
       </c>
       <c r="H341" t="str">
-        <f t="shared" ref="H341:H342" si="1">SUBSTITUTE(G341,"_"," ")</f>
+        <f t="shared" ref="H341:H342" si="2">SUBSTITUTE(G341,"_"," ")</f>
         <v>kosam sultan</v>
       </c>
     </row>
@@ -5726,7 +5693,7 @@
         <v>443</v>
       </c>
       <c r="H342" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>sultan ahmad</v>
       </c>
     </row>
@@ -5740,26 +5707,36 @@
       <c r="B344" t="s">
         <v>440</v>
       </c>
+      <c r="E344" t="str">
+        <f>SUBSTITUTE(B339,D339,C339)</f>
+        <v>old text</v>
+      </c>
+    </row>
+    <row r="345" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F345" t="str">
+        <f>SUBSTITUTE(B339," ","   ")</f>
+        <v>old   text</v>
+      </c>
     </row>
     <row r="346" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B346" s="50" t="s">
+      <c r="B346" s="52" t="s">
         <v>195</v>
       </c>
-      <c r="C346" s="49"/>
-      <c r="D346" s="49"/>
-      <c r="E346" s="49"/>
+      <c r="C346" s="51"/>
+      <c r="D346" s="51"/>
+      <c r="E346" s="51"/>
     </row>
     <row r="347" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B347" s="49"/>
-      <c r="C347" s="49"/>
-      <c r="D347" s="49"/>
-      <c r="E347" s="49"/>
+      <c r="B347" s="51"/>
+      <c r="C347" s="51"/>
+      <c r="D347" s="51"/>
+      <c r="E347" s="51"/>
     </row>
     <row r="348" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B348" s="49"/>
-      <c r="C348" s="49"/>
-      <c r="D348" s="49"/>
-      <c r="E348" s="49"/>
+      <c r="B348" s="51"/>
+      <c r="C348" s="51"/>
+      <c r="D348" s="51"/>
+      <c r="E348" s="51"/>
     </row>
     <row r="350" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B350" t="s">
@@ -5845,11 +5822,11 @@
         <v>fail</v>
       </c>
       <c r="E362" t="str">
-        <f t="shared" ref="E362:E367" si="2">IF(AND(B362&gt;60,C362="CS"),"give","not give")</f>
+        <f t="shared" ref="E362:E367" si="3">IF(AND(B362&gt;60,C362="CS"),"give","not give")</f>
         <v>not give</v>
       </c>
       <c r="F362" t="str">
-        <f t="shared" ref="F362:F367" si="3">IF(AND(B362&gt;50, C362="CS"), "ELI","NON")</f>
+        <f t="shared" ref="F362:F367" si="4">IF(AND(B362&gt;50, C362="CS"), "ELI","NON")</f>
         <v>NON</v>
       </c>
     </row>
@@ -5861,15 +5838,15 @@
         <v>198</v>
       </c>
       <c r="D363" t="str">
-        <f t="shared" ref="D363:D367" si="4">IF(B363&gt;50,"pass","fail")</f>
+        <f t="shared" ref="D363:D367" si="5">IF(B363&gt;50,"pass","fail")</f>
         <v>pass</v>
       </c>
       <c r="E363" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>give</v>
       </c>
       <c r="F363" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>ELI</v>
       </c>
     </row>
@@ -5881,15 +5858,15 @@
         <v>200</v>
       </c>
       <c r="D364" t="str">
+        <f t="shared" si="5"/>
+        <v>fail</v>
+      </c>
+      <c r="E364" t="str">
+        <f t="shared" si="3"/>
+        <v>not give</v>
+      </c>
+      <c r="F364" t="str">
         <f t="shared" si="4"/>
-        <v>fail</v>
-      </c>
-      <c r="E364" t="str">
-        <f t="shared" si="2"/>
-        <v>not give</v>
-      </c>
-      <c r="F364" t="str">
-        <f t="shared" si="3"/>
         <v>NON</v>
       </c>
     </row>
@@ -5901,15 +5878,15 @@
         <v>200</v>
       </c>
       <c r="D365" t="str">
+        <f t="shared" si="5"/>
+        <v>pass</v>
+      </c>
+      <c r="E365" t="str">
+        <f t="shared" si="3"/>
+        <v>not give</v>
+      </c>
+      <c r="F365" t="str">
         <f t="shared" si="4"/>
-        <v>pass</v>
-      </c>
-      <c r="E365" t="str">
-        <f t="shared" si="2"/>
-        <v>not give</v>
-      </c>
-      <c r="F365" t="str">
-        <f t="shared" si="3"/>
         <v>NON</v>
       </c>
     </row>
@@ -5921,15 +5898,15 @@
         <v>199</v>
       </c>
       <c r="D366" t="str">
+        <f t="shared" si="5"/>
+        <v>pass</v>
+      </c>
+      <c r="E366" t="str">
+        <f t="shared" si="3"/>
+        <v>not give</v>
+      </c>
+      <c r="F366" t="str">
         <f t="shared" si="4"/>
-        <v>pass</v>
-      </c>
-      <c r="E366" t="str">
-        <f t="shared" si="2"/>
-        <v>not give</v>
-      </c>
-      <c r="F366" t="str">
-        <f t="shared" si="3"/>
         <v>NON</v>
       </c>
     </row>
@@ -5941,27 +5918,27 @@
         <v>199</v>
       </c>
       <c r="D367" t="str">
+        <f t="shared" si="5"/>
+        <v>pass</v>
+      </c>
+      <c r="E367" t="str">
+        <f t="shared" si="3"/>
+        <v>not give</v>
+      </c>
+      <c r="F367" t="str">
         <f t="shared" si="4"/>
-        <v>pass</v>
-      </c>
-      <c r="E367" t="str">
-        <f t="shared" si="2"/>
-        <v>not give</v>
-      </c>
-      <c r="F367" t="str">
-        <f t="shared" si="3"/>
         <v>NON</v>
       </c>
     </row>
     <row r="370" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C370" s="56" t="s">
+      <c r="C370" s="58" t="s">
         <v>210</v>
       </c>
-      <c r="D370" s="56"/>
+      <c r="D370" s="58"/>
     </row>
     <row r="371" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C371" s="56"/>
-      <c r="D371" s="56"/>
+      <c r="C371" s="58"/>
+      <c r="D371" s="58"/>
     </row>
     <row r="373" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B373" t="s">
@@ -6011,7 +5988,7 @@
         <v>5</v>
       </c>
       <c r="D378" t="str">
-        <f t="shared" ref="D378:D384" si="5">IF(AND(B378=1,C378=0),"single",IF(AND(B378=2,C378=0),"couple","family"))</f>
+        <f t="shared" ref="D378:D384" si="6">IF(AND(B378=1,C378=0),"single",IF(AND(B378=2,C378=0),"couple","family"))</f>
         <v>family</v>
       </c>
       <c r="F378" t="s">
@@ -6026,7 +6003,7 @@
         <v>0</v>
       </c>
       <c r="D379" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>single</v>
       </c>
     </row>
@@ -6038,7 +6015,7 @@
         <v>3</v>
       </c>
       <c r="D380" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>family</v>
       </c>
     </row>
@@ -6050,7 +6027,7 @@
         <v>1</v>
       </c>
       <c r="D381" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>family</v>
       </c>
     </row>
@@ -6062,7 +6039,7 @@
         <v>0</v>
       </c>
       <c r="D382" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>couple</v>
       </c>
     </row>
@@ -6074,7 +6051,7 @@
         <v>3</v>
       </c>
       <c r="D383" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>family</v>
       </c>
     </row>
@@ -6086,29 +6063,29 @@
         <v>0</v>
       </c>
       <c r="D384" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>single</v>
       </c>
     </row>
     <row r="386" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B386" s="50" t="s">
+      <c r="B386" s="52" t="s">
         <v>219</v>
       </c>
-      <c r="C386" s="49"/>
-      <c r="D386" s="49"/>
-      <c r="E386" s="49"/>
+      <c r="C386" s="51"/>
+      <c r="D386" s="51"/>
+      <c r="E386" s="51"/>
     </row>
     <row r="387" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B387" s="49"/>
-      <c r="C387" s="49"/>
-      <c r="D387" s="49"/>
-      <c r="E387" s="49"/>
+      <c r="B387" s="51"/>
+      <c r="C387" s="51"/>
+      <c r="D387" s="51"/>
+      <c r="E387" s="51"/>
     </row>
     <row r="388" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B388" s="49"/>
-      <c r="C388" s="49"/>
-      <c r="D388" s="49"/>
-      <c r="E388" s="49"/>
+      <c r="B388" s="51"/>
+      <c r="C388" s="51"/>
+      <c r="D388" s="51"/>
+      <c r="E388" s="51"/>
     </row>
     <row r="390" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B390" t="s">
@@ -6116,7 +6093,7 @@
       </c>
       <c r="C390" s="8">
         <f ca="1">TODAY()</f>
-        <v>46149</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="391" spans="2:5" x14ac:dyDescent="0.35">
@@ -6125,7 +6102,7 @@
       </c>
       <c r="C391" s="22">
         <f ca="1">NOW()</f>
-        <v>46149.481748611113</v>
+        <v>46189.577346874998</v>
       </c>
     </row>
     <row r="392" spans="2:5" x14ac:dyDescent="0.35">
@@ -6134,7 +6111,7 @@
       </c>
       <c r="C392">
         <f ca="1">SECOND(C391)</f>
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="D392" t="s">
         <v>223</v>
@@ -6146,7 +6123,7 @@
       </c>
       <c r="C393">
         <f ca="1">MINUTE(C391)</f>
-        <v>33</v>
+        <v>51</v>
       </c>
     </row>
     <row r="394" spans="2:5" x14ac:dyDescent="0.35">
@@ -6155,7 +6132,7 @@
       </c>
       <c r="C394">
         <f ca="1">HOUR(C391)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="395" spans="2:5" x14ac:dyDescent="0.35">
@@ -6164,7 +6141,7 @@
       </c>
       <c r="C395">
         <f ca="1">DAY(C391)</f>
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="396" spans="2:5" x14ac:dyDescent="0.35">
@@ -6173,7 +6150,7 @@
       </c>
       <c r="C396">
         <f ca="1">MONTH(C391)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="397" spans="2:5" x14ac:dyDescent="0.35">
@@ -6215,7 +6192,7 @@
     <row r="403" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C403" s="8">
         <f ca="1">EDATE(C390,2)</f>
-        <v>46210</v>
+        <v>46250</v>
       </c>
     </row>
     <row r="405" spans="2:8" x14ac:dyDescent="0.35">
@@ -6226,38 +6203,42 @@
     <row r="406" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C406" s="8">
         <f ca="1">EDATE(C390,2*12)</f>
-        <v>46880</v>
+        <v>46920</v>
       </c>
     </row>
     <row r="408" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B408" s="50" t="s">
+      <c r="B408" s="52" t="s">
         <v>232</v>
       </c>
-      <c r="C408" s="49"/>
-      <c r="D408" s="49"/>
-      <c r="E408" s="49"/>
+      <c r="C408" s="51"/>
+      <c r="D408" s="51"/>
+      <c r="E408" s="51"/>
     </row>
     <row r="409" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B409" s="49"/>
-      <c r="C409" s="49"/>
-      <c r="D409" s="49"/>
-      <c r="E409" s="49"/>
+      <c r="B409" s="51"/>
+      <c r="C409" s="51"/>
+      <c r="D409" s="51"/>
+      <c r="E409" s="51"/>
     </row>
     <row r="410" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B410" s="49"/>
-      <c r="C410" s="49"/>
-      <c r="D410" s="49"/>
-      <c r="E410" s="49"/>
+      <c r="B410" s="51"/>
+      <c r="C410" s="51"/>
+      <c r="D410" s="51"/>
+      <c r="E410" s="51"/>
       <c r="F410">
-        <f>COUNTIFS(Table510[AMOUNT],"&gt;1",Table510[SUB-CATEGORY],"kapry")</f>
-        <v>1</v>
+        <f>COUNTIFS(Table510[AMOUNT],"&gt;5",Table510[SUB-CATEGORY],"chai")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="411" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B411" s="49"/>
-      <c r="C411" s="49"/>
-      <c r="D411" s="49"/>
-      <c r="E411" s="49"/>
+      <c r="B411" s="51"/>
+      <c r="C411" s="51"/>
+      <c r="D411" s="51"/>
+      <c r="E411" s="51"/>
+      <c r="H411">
+        <f>COUNTIF(Table510[AMOUNT],D415)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="412" spans="2:8" x14ac:dyDescent="0.35">
       <c r="E412">
@@ -6352,9 +6333,11 @@
       <c r="E418" s="17">
         <v>4</v>
       </c>
-      <c r="G418" t="s">
+      <c r="G418" s="45" t="s">
         <v>235</v>
       </c>
+      <c r="H418" s="45"/>
+      <c r="I418" s="45"/>
     </row>
     <row r="419" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B419" s="8">
@@ -6369,9 +6352,11 @@
       <c r="E419" s="17">
         <v>5</v>
       </c>
-      <c r="G419" t="s">
+      <c r="G419" s="45" t="s">
         <v>237</v>
       </c>
+      <c r="H419" s="45"/>
+      <c r="I419" s="45"/>
     </row>
     <row r="420" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B420" s="8">
@@ -6386,9 +6371,11 @@
       <c r="E420" s="17">
         <v>6</v>
       </c>
-      <c r="G420" t="s">
+      <c r="G420" s="45" t="s">
         <v>236</v>
       </c>
+      <c r="H420" s="45"/>
+      <c r="I420" s="45"/>
     </row>
     <row r="421" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B421" s="8">
@@ -6403,9 +6390,11 @@
       <c r="E421" s="17">
         <v>7</v>
       </c>
-      <c r="G421" t="s">
+      <c r="G421" s="45" t="s">
         <v>239</v>
       </c>
+      <c r="H421" s="45"/>
+      <c r="I421" s="45"/>
     </row>
     <row r="422" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B422" s="8">
@@ -6420,9 +6409,11 @@
       <c r="E422" s="17">
         <v>8</v>
       </c>
-      <c r="G422" t="s">
+      <c r="G422" s="45" t="s">
         <v>238</v>
       </c>
+      <c r="H422" s="45"/>
+      <c r="I422" s="45"/>
     </row>
     <row r="423" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B423" s="8">
@@ -6634,34 +6625,34 @@
       </c>
     </row>
     <row r="440" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B440" s="50" t="s">
+      <c r="B440" s="52" t="s">
         <v>259</v>
       </c>
-      <c r="C440" s="49"/>
-      <c r="D440" s="49"/>
-      <c r="E440" s="49"/>
-      <c r="F440" s="49"/>
+      <c r="C440" s="51"/>
+      <c r="D440" s="51"/>
+      <c r="E440" s="51"/>
+      <c r="F440" s="51"/>
     </row>
     <row r="441" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B441" s="49"/>
-      <c r="C441" s="49"/>
-      <c r="D441" s="49"/>
-      <c r="E441" s="49"/>
-      <c r="F441" s="49"/>
+      <c r="B441" s="51"/>
+      <c r="C441" s="51"/>
+      <c r="D441" s="51"/>
+      <c r="E441" s="51"/>
+      <c r="F441" s="51"/>
     </row>
     <row r="442" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B442" s="49"/>
-      <c r="C442" s="49"/>
-      <c r="D442" s="49"/>
-      <c r="E442" s="49"/>
-      <c r="F442" s="49"/>
+      <c r="B442" s="51"/>
+      <c r="C442" s="51"/>
+      <c r="D442" s="51"/>
+      <c r="E442" s="51"/>
+      <c r="F442" s="51"/>
     </row>
     <row r="443" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B443" s="49"/>
-      <c r="C443" s="49"/>
-      <c r="D443" s="49"/>
-      <c r="E443" s="49"/>
-      <c r="F443" s="49"/>
+      <c r="B443" s="51"/>
+      <c r="C443" s="51"/>
+      <c r="D443" s="51"/>
+      <c r="E443" s="51"/>
+      <c r="F443" s="51"/>
     </row>
     <row r="445" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B445" s="29"/>
@@ -6700,6 +6691,10 @@
         <f>LOOKUP(B448,F448:F453,G448:G453)</f>
         <v>F</v>
       </c>
+      <c r="E448" t="str">
+        <f>LOOKUP(B448,$F$448:$F$453,$G$448:$G$453)</f>
+        <v>F</v>
+      </c>
       <c r="F448">
         <v>0</v>
       </c>
@@ -6712,13 +6707,17 @@
         <v>56</v>
       </c>
       <c r="C449" t="str">
-        <f t="shared" ref="C449:C455" si="6">IF(B449&gt;=50,"pass","fail")</f>
+        <f t="shared" ref="C449:C455" si="7">IF(B449&gt;=50,"pass","fail")</f>
         <v>pass</v>
       </c>
       <c r="D449" t="str">
         <f>LOOKUP(B449,F449:F454,G449:G454)</f>
         <v>D</v>
       </c>
+      <c r="E449" t="str">
+        <f t="shared" ref="E449:E455" si="8">LOOKUP(B449,$F$448:$F$453,$G$448:$G$453)</f>
+        <v>D</v>
+      </c>
       <c r="F449">
         <v>50</v>
       </c>
@@ -6731,13 +6730,17 @@
         <v>98</v>
       </c>
       <c r="C450" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>pass</v>
       </c>
       <c r="D450" t="str">
         <f>LOOKUP(B450,F450:F455,G450:G455)</f>
         <v>A+</v>
       </c>
+      <c r="E450" t="str">
+        <f t="shared" si="8"/>
+        <v>A+</v>
+      </c>
       <c r="F450">
         <v>60</v>
       </c>
@@ -6753,13 +6756,17 @@
         <v>24</v>
       </c>
       <c r="C451" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>fail</v>
       </c>
       <c r="D451" t="e">
         <f>LOOKUP(B451,F451:F456,G451:G456)</f>
         <v>#N/A</v>
       </c>
+      <c r="E451" t="str">
+        <f t="shared" si="8"/>
+        <v>F</v>
+      </c>
       <c r="F451">
         <v>70</v>
       </c>
@@ -6775,12 +6782,16 @@
         <v>71</v>
       </c>
       <c r="C452" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>pass</v>
       </c>
       <c r="D452" t="e">
-        <f t="shared" ref="D452:D455" si="7">LOOKUP(B452,F452:F457,G452:G457)</f>
+        <f t="shared" ref="D452:D455" si="9">LOOKUP(B452,F452:F457,G452:G457)</f>
         <v>#N/A</v>
+      </c>
+      <c r="E452" t="str">
+        <f t="shared" si="8"/>
+        <v>B</v>
       </c>
       <c r="F452">
         <v>80</v>
@@ -6797,12 +6808,16 @@
         <v>89</v>
       </c>
       <c r="C453" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>pass</v>
       </c>
       <c r="D453" t="e">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>#N/A</v>
+      </c>
+      <c r="E453" t="str">
+        <f t="shared" si="8"/>
+        <v>A+</v>
       </c>
       <c r="F453">
         <v>90</v>
@@ -6823,8 +6838,12 @@
         <v>fail</v>
       </c>
       <c r="D454" t="e">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>#N/A</v>
+      </c>
+      <c r="E454" t="str">
+        <f t="shared" si="8"/>
+        <v>F</v>
       </c>
       <c r="H454" t="s">
         <v>454</v>
@@ -6835,12 +6854,16 @@
         <v>78</v>
       </c>
       <c r="C455" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>pass</v>
       </c>
       <c r="D455" t="e">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>#N/A</v>
+      </c>
+      <c r="E455" t="str">
+        <f t="shared" si="8"/>
+        <v>B</v>
       </c>
       <c r="H455" t="s">
         <v>455</v>
@@ -6955,7 +6978,7 @@
         <v>447</v>
       </c>
       <c r="J464" s="45" t="str">
-        <f t="shared" ref="J464:J465" ca="1" si="8">LOOKUP(I464,$L$461:$L$464,$M$461)</f>
+        <f t="shared" ref="J464:J465" ca="1" si="10">LOOKUP(I464,$L$461:$L$464,$M$461)</f>
         <v>USA</v>
       </c>
       <c r="K464" s="45"/>
@@ -6989,7 +7012,7 @@
         <v>449</v>
       </c>
       <c r="J465" s="45" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="10"/>
         <v>USA</v>
       </c>
       <c r="K465" s="45"/>
@@ -7002,7 +7025,7 @@
         <v>56</v>
       </c>
       <c r="C466" t="str">
-        <f t="shared" ref="C466:C472" si="9">IF(B466&gt;=50,"pass","fail")</f>
+        <f t="shared" ref="C466:C472" si="11">IF(B466&gt;=50,"pass","fail")</f>
         <v>pass</v>
       </c>
       <c r="D466" t="str">
@@ -7023,11 +7046,11 @@
         <v>98</v>
       </c>
       <c r="C467" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>pass</v>
       </c>
       <c r="D467" t="str">
-        <f t="shared" ref="D467:D472" si="10">LOOKUP(B467,$F$465:$F$470,$G$465:$G$470)</f>
+        <f t="shared" ref="D467:D472" si="12">LOOKUP(B467,$F$465:$F$470,$G$465:$G$470)</f>
         <v>A+</v>
       </c>
       <c r="F467">
@@ -7042,11 +7065,11 @@
         <v>24</v>
       </c>
       <c r="C468" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>fail</v>
       </c>
       <c r="D468" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>F</v>
       </c>
       <c r="F468">
@@ -7064,11 +7087,11 @@
         <v>71</v>
       </c>
       <c r="C469" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>pass</v>
       </c>
       <c r="D469" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>B</v>
       </c>
       <c r="F469">
@@ -7086,11 +7109,11 @@
         <v>89</v>
       </c>
       <c r="C470" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>pass</v>
       </c>
       <c r="D470" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>A+</v>
       </c>
       <c r="F470">
@@ -7108,11 +7131,11 @@
         <v>46</v>
       </c>
       <c r="C471" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>fail</v>
       </c>
       <c r="D471" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>F</v>
       </c>
       <c r="J471" t="s">
@@ -7124,11 +7147,11 @@
         <v>78</v>
       </c>
       <c r="C472" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>pass</v>
       </c>
       <c r="D472" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>B</v>
       </c>
     </row>
@@ -7197,7 +7220,7 @@
         <v>100000</v>
       </c>
       <c r="E481" s="28">
-        <f t="shared" ref="E481:E486" si="11">LOOKUP(D481,$G$480:$G$483,$H$480:$H$483)</f>
+        <f t="shared" ref="E481:E486" si="13">LOOKUP(D481,$G$480:$G$483,$H$480:$H$483)</f>
         <v>0.5</v>
       </c>
       <c r="G481" s="26">
@@ -7218,7 +7241,7 @@
         <v>130000</v>
       </c>
       <c r="E482" s="28">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0.5</v>
       </c>
       <c r="G482" s="26">
@@ -7239,7 +7262,7 @@
         <v>68000</v>
       </c>
       <c r="E483" s="28">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0.2</v>
       </c>
       <c r="G483" s="26">
@@ -7260,7 +7283,7 @@
         <v>100000</v>
       </c>
       <c r="E484" s="28">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0.5</v>
       </c>
     </row>
@@ -7275,7 +7298,7 @@
         <v>56000</v>
       </c>
       <c r="E485" s="28">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0.2</v>
       </c>
     </row>
@@ -7290,12 +7313,12 @@
         <v>90000</v>
       </c>
       <c r="E486" s="28">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0.2</v>
       </c>
     </row>
     <row r="488" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B488" s="55" t="s">
+      <c r="B488" s="57" t="s">
         <v>283</v>
       </c>
       <c r="D488" t="str">
@@ -7304,7 +7327,7 @@
       </c>
     </row>
     <row r="489" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B489" s="55"/>
+      <c r="B489" s="57"/>
       <c r="C489" t="s">
         <v>284</v>
       </c>
@@ -7539,22 +7562,22 @@
         <v>331</v>
       </c>
     </row>
-    <row r="513" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="513" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C513" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="514" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="514" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C514" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="515" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="515" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C515" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="519" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B519" t="e">
         <f>VLOOKUP(D498,Table7[#All],2,FALSE)</f>
         <v>#N/A</v>
@@ -7563,7 +7586,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="521" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="521" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B521" t="e">
         <f>VLOOKUP(C492,Table7[#All],3,FALSE)</f>
         <v>#N/A</v>
@@ -7572,7 +7595,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="523" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="523" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B523">
         <f>VLOOKUP(C492,Table7[[#All],[NAME]:[GENDER]],2,FALSE)</f>
         <v>54</v>
@@ -7581,7 +7604,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="526" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="526" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A526" t="s">
         <v>275</v>
       </c>
@@ -7598,7 +7621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="527" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A527" t="s">
         <v>311</v>
       </c>
@@ -7612,7 +7635,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="528" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="528" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A528" t="s">
         <v>265</v>
       </c>
@@ -7625,8 +7648,12 @@
       <c r="D528" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="529" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F528" t="str">
+        <f>VLOOKUP(B528,B527:D537,3,)</f>
+        <v>india</v>
+      </c>
+    </row>
+    <row r="529" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A529" t="s">
         <v>265</v>
       </c>
@@ -7640,7 +7667,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="530" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="530" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A530" t="s">
         <v>265</v>
       </c>
@@ -7657,8 +7684,13 @@
         <f>VLOOKUP(B528,B526:D537,2)</f>
         <v>11</v>
       </c>
-    </row>
-    <row r="531" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G530" s="45"/>
+      <c r="H530" s="45"/>
+      <c r="I530" s="45"/>
+      <c r="J530" s="45"/>
+      <c r="K530" s="45"/>
+    </row>
+    <row r="531" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A531" t="s">
         <v>312</v>
       </c>
@@ -7675,8 +7707,15 @@
         <f>VLOOKUP(A528,A527:D537,3)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="532" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G531" s="45" t="s">
+        <v>468</v>
+      </c>
+      <c r="H531" s="45"/>
+      <c r="I531" s="45"/>
+      <c r="J531" s="45"/>
+      <c r="K531" s="45"/>
+    </row>
+    <row r="532" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A532" t="s">
         <v>13</v>
       </c>
@@ -7689,8 +7728,15 @@
       <c r="D532" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="533" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G532" s="45" t="s">
+        <v>469</v>
+      </c>
+      <c r="H532" s="45"/>
+      <c r="I532" s="45"/>
+      <c r="J532" s="45"/>
+      <c r="K532" s="45"/>
+    </row>
+    <row r="533" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A533" t="s">
         <v>313</v>
       </c>
@@ -7711,8 +7757,13 @@
         <f>VLOOKUP(A528,A526:D537,2)</f>
         <v>b</v>
       </c>
-    </row>
-    <row r="534" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G533" s="45"/>
+      <c r="H533" s="45"/>
+      <c r="I533" s="45"/>
+      <c r="J533" s="45"/>
+      <c r="K533" s="45"/>
+    </row>
+    <row r="534" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A534" t="s">
         <v>314</v>
       </c>
@@ -7730,7 +7781,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="535" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="535" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A535" t="s">
         <v>315</v>
       </c>
@@ -7748,7 +7799,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="536" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
         <v>316</v>
       </c>
@@ -7762,7 +7813,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="537" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="537" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A537" t="s">
         <v>317</v>
       </c>
@@ -7776,41 +7827,41 @@
         <v>320</v>
       </c>
     </row>
-    <row r="538" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="538" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E538" t="str">
         <f>INDEX(D527:D537,MATCH(B528,B527:B537))</f>
         <v>pak</v>
       </c>
     </row>
-    <row r="541" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B541" s="50" t="s">
+    <row r="541" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B541" s="52" t="s">
         <v>333</v>
       </c>
-      <c r="C541" s="49"/>
-      <c r="D541" s="49"/>
-      <c r="E541" s="49"/>
-      <c r="F541" s="49"/>
-    </row>
-    <row r="542" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B542" s="49"/>
-      <c r="C542" s="49"/>
-      <c r="D542" s="49"/>
-      <c r="E542" s="49"/>
-      <c r="F542" s="49"/>
-    </row>
-    <row r="543" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B543" s="49"/>
-      <c r="C543" s="49"/>
-      <c r="D543" s="49"/>
-      <c r="E543" s="49"/>
-      <c r="F543" s="49"/>
-    </row>
-    <row r="544" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B544" s="49"/>
-      <c r="C544" s="49"/>
-      <c r="D544" s="49"/>
-      <c r="E544" s="49"/>
-      <c r="F544" s="49"/>
+      <c r="C541" s="51"/>
+      <c r="D541" s="51"/>
+      <c r="E541" s="51"/>
+      <c r="F541" s="51"/>
+    </row>
+    <row r="542" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B542" s="51"/>
+      <c r="C542" s="51"/>
+      <c r="D542" s="51"/>
+      <c r="E542" s="51"/>
+      <c r="F542" s="51"/>
+    </row>
+    <row r="543" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B543" s="51"/>
+      <c r="C543" s="51"/>
+      <c r="D543" s="51"/>
+      <c r="E543" s="51"/>
+      <c r="F543" s="51"/>
+    </row>
+    <row r="544" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B544" s="51"/>
+      <c r="C544" s="51"/>
+      <c r="D544" s="51"/>
+      <c r="E544" s="51"/>
+      <c r="F544" s="51"/>
     </row>
     <row r="545" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C545" t="s">
@@ -8024,7 +8075,13 @@
         <v>140</v>
       </c>
     </row>
-    <row r="562" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="561" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G561" t="str">
+        <f>_xlfn.XLOOKUP(C551,Table79[NAME],Table79[ID])</f>
+        <v>A1003</v>
+      </c>
+    </row>
+    <row r="562" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B562">
         <f>B565</f>
         <v>0</v>
@@ -8037,26 +8094,30 @@
         <f>_xlfn.XLOOKUP(D551,Table79[AGE],Table79[ID])</f>
         <v>A1003</v>
       </c>
-    </row>
-    <row r="563" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="G562">
+        <f>_xlfn.XLOOKUP(C551,Table79[NAME],Table79[AGE],,,-1)</f>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="563" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C563" t="str">
         <f>INDEX(Table79[GENDER],MATCH(B552,Table79[ID]))</f>
         <v>M</v>
       </c>
     </row>
-    <row r="564" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="564" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E564">
         <f>_xlfn.XLOOKUP(B552,Table79[ID],Table79[AGE])</f>
         <v>221</v>
       </c>
     </row>
-    <row r="565" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="565" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C565">
         <f>VLOOKUP(B552,Table79[],3)</f>
         <v>221</v>
       </c>
     </row>
-    <row r="570" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="570" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B570" s="24" t="s">
         <v>339</v>
       </c>
@@ -8065,22 +8126,22 @@
       </c>
       <c r="D570" s="45"/>
     </row>
-    <row r="571" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="571" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C571" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="572" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="572" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C572" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="573" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="573" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C573" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="575" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="575" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C575" t="str">
         <f>INDEX(Table79[ID],5,1)</f>
         <v>A1005</v>
@@ -8180,30 +8241,30 @@
       <c r="G592" s="32"/>
     </row>
     <row r="594" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B594" s="50" t="s">
+      <c r="B594" s="52" t="s">
         <v>359</v>
       </c>
-      <c r="C594" s="49"/>
-      <c r="D594" s="49"/>
-      <c r="E594" s="49"/>
+      <c r="C594" s="51"/>
+      <c r="D594" s="51"/>
+      <c r="E594" s="51"/>
     </row>
     <row r="595" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B595" s="49"/>
-      <c r="C595" s="49"/>
-      <c r="D595" s="49"/>
-      <c r="E595" s="49"/>
+      <c r="B595" s="51"/>
+      <c r="C595" s="51"/>
+      <c r="D595" s="51"/>
+      <c r="E595" s="51"/>
     </row>
     <row r="596" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B596" s="49"/>
-      <c r="C596" s="49"/>
-      <c r="D596" s="49"/>
-      <c r="E596" s="49"/>
+      <c r="B596" s="51"/>
+      <c r="C596" s="51"/>
+      <c r="D596" s="51"/>
+      <c r="E596" s="51"/>
     </row>
     <row r="597" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B597" s="49"/>
-      <c r="C597" s="49"/>
-      <c r="D597" s="49"/>
-      <c r="E597" s="49"/>
+      <c r="B597" s="51"/>
+      <c r="C597" s="51"/>
+      <c r="D597" s="51"/>
+      <c r="E597" s="51"/>
     </row>
     <row r="599" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B599" t="s">
@@ -8247,30 +8308,30 @@
       </c>
     </row>
     <row r="607" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B607" s="50" t="s">
+      <c r="B607" s="52" t="s">
         <v>367</v>
       </c>
-      <c r="C607" s="49"/>
-      <c r="D607" s="49"/>
-      <c r="E607" s="49"/>
+      <c r="C607" s="51"/>
+      <c r="D607" s="51"/>
+      <c r="E607" s="51"/>
     </row>
     <row r="608" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B608" s="49"/>
-      <c r="C608" s="49"/>
-      <c r="D608" s="49"/>
-      <c r="E608" s="49"/>
+      <c r="B608" s="51"/>
+      <c r="C608" s="51"/>
+      <c r="D608" s="51"/>
+      <c r="E608" s="51"/>
     </row>
     <row r="609" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B609" s="49"/>
-      <c r="C609" s="49"/>
-      <c r="D609" s="49"/>
-      <c r="E609" s="49"/>
+      <c r="B609" s="51"/>
+      <c r="C609" s="51"/>
+      <c r="D609" s="51"/>
+      <c r="E609" s="51"/>
     </row>
     <row r="610" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B610" s="49"/>
-      <c r="C610" s="49"/>
-      <c r="D610" s="49"/>
-      <c r="E610" s="49"/>
+      <c r="B610" s="51"/>
+      <c r="C610" s="51"/>
+      <c r="D610" s="51"/>
+      <c r="E610" s="51"/>
     </row>
     <row r="612" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B612" t="s">
@@ -8362,7 +8423,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B180:B187">
-    <cfRule type="timePeriod" dxfId="7" priority="6" timePeriod="lastMonth">
+    <cfRule type="timePeriod" dxfId="4" priority="6" timePeriod="lastMonth">
       <formula>AND(MONTH(B180)=MONTH(EDATE(TODAY(),0-1)),YEAR(B180)=YEAR(EDATE(TODAY(),0-1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8381,7 +8442,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D106:D113">
-    <cfRule type="containsText" dxfId="6" priority="24" operator="containsText" text="oo">
+    <cfRule type="containsText" dxfId="3" priority="24" operator="containsText" text="oo">
       <formula>NOT(ISERROR(SEARCH("oo",D106)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8407,7 +8468,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E106:E113">
-    <cfRule type="cellIs" dxfId="5" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
       <formula>"phone"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8424,16 +8485,16 @@
         </ext>
       </extLst>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="25" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="25" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J78:J82">
-    <cfRule type="containsText" dxfId="3" priority="9" operator="containsText" text="n">
+    <cfRule type="containsText" dxfId="0" priority="9" operator="containsText" text="n">
       <formula>NOT(ISERROR(SEARCH("n",J78)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="6">
+  <dataValidations count="7">
     <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B78:B82 B179 C105:C113" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>45261</formula1>
       <formula2>45290</formula2>
@@ -8453,6 +8514,10 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D78:D82" xr:uid="{CF6F91F0-AD84-497A-915C-933E775732C2}">
       <formula1>"PHONE, TABLE"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E79:E82" xr:uid="{3C089A3F-C88F-4BEA-9C73-80327A369CF3}">
+      <formula1>10</formula1>
+      <formula2>800</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>